<commit_message>
feat: add register reference documentation generation
- Introduced CSS and JS files for styling and functionality of the register reference documentation.
- Implemented HTML template for rendering register documentation with dynamic content.
- Created Rust modules for handling anchor ID generation, error management, HTML serialization, and view models for components, blocks, registers, and fields.
- Added functionality to search registers and toggle between light and dark themes.
- Developed tests to ensure correct serialization of register documentation and handling of register files.
</commit_message>
<xml_diff>
--- a/crates/snapsheet/tests/fixtures/conflicting_registers.xlsx
+++ b/crates/snapsheet/tests/fixtures/conflicting_registers.xlsx
@@ -117,19 +117,19 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>REG_DESC</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>FIELD</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>BIT</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>WIDTH</t>
-        </is>
-      </c>
       <c r="F1" t="inlineStr">
         <is>
           <t>ATTRIBUTE</t>
@@ -142,7 +142,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>DESCRIPTION</t>
+          <t>FIELD_DESC</t>
         </is>
       </c>
     </row>
@@ -157,19 +157,14 @@
           <t>reg</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>[31:0]</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>32</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -194,19 +189,14 @@
           <t>reg</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>[31:0]</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>32</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">

</xml_diff>

<commit_message>
feat: Refactor register handling and documentation generation
- Introduced `RegisterSource` enum to differentiate between direct registers and register files.
- Updated `RegisterView` to include source information.
- Enhanced register file parsing to support multiple instances and offsets.
- Modified HTML templates for register and block references to improve structure and styling.
- Updated configuration to include descriptions for version and address block columns.
- Changed column headers in snapsheet format from `ATTRIBUTE` and `DEFAULT` to `ATTR` and `RESET`.
- Added new templates for detailed register views and block references.
- Improved documentation regarding RALF and SystemRDL output behaviors.
- Updated tests and fixtures to reflect changes in register naming and structure.
</commit_message>
<xml_diff>
--- a/crates/snapsheet/tests/fixtures/conflicting_registers.xlsx
+++ b/crates/snapsheet/tests/fixtures/conflicting_registers.xlsx
@@ -132,12 +132,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>ATTRIBUTE</t>
+          <t>ATTR</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>DEFAULT</t>
+          <t>RESET</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">

</xml_diff>